<commit_message>
feat: Add Complete Master CI/CD and Automation Suite
</commit_message>
<xml_diff>
--- a/Vulnerability Test Results/endpoint-inventory.xlsx
+++ b/Vulnerability Test Results/endpoint-inventory.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Endpoints" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Endpoint Inventory" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
   <si>
     <t>Endpoint</t>
   </si>
@@ -19,13 +19,19 @@
     <t>HTTP Method</t>
   </si>
   <si>
-    <t>Authentication Required</t>
+    <t>Auth Required</t>
   </si>
   <si>
     <t>Expected Roles</t>
   </si>
   <si>
-    <t>/auth/register</t>
+    <t>Controller</t>
+  </si>
+  <si>
+    <t>Source File</t>
+  </si>
+  <si>
+    <t>/api/auth/login</t>
   </si>
   <si>
     <t>POST</t>
@@ -34,16 +40,28 @@
     <t>No</t>
   </si>
   <si>
-    <t>Public</t>
-  </si>
-  <si>
-    <t>/auth/login</t>
-  </si>
-  <si>
-    <t>/auth/verify-email</t>
-  </si>
-  <si>
-    <t>/auth/me</t>
+    <t>Any</t>
+  </si>
+  <si>
+    <t>loginController</t>
+  </si>
+  <si>
+    <t>routes/auth.js</t>
+  </si>
+  <si>
+    <t>/api/auth/register</t>
+  </si>
+  <si>
+    <t>registerController</t>
+  </si>
+  <si>
+    <t>/api/auth/forgot-password</t>
+  </si>
+  <si>
+    <t>forgotPassword</t>
+  </si>
+  <si>
+    <t>/api/users/profile/:id</t>
   </si>
   <si>
     <t>GET</t>
@@ -52,34 +70,34 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>User</t>
-  </si>
-  <si>
-    <t>/auth/forgot-password</t>
-  </si>
-  <si>
-    <t>/auth/reset-password</t>
-  </si>
-  <si>
-    <t>/user/export</t>
-  </si>
-  <si>
-    <t>/auth/2fa/generate</t>
-  </si>
-  <si>
-    <t>/auth/2fa/verify</t>
-  </si>
-  <si>
-    <t>/analyze-document</t>
-  </si>
-  <si>
-    <t>/analyze-url</t>
-  </si>
-  <si>
-    <t>/feed</t>
-  </si>
-  <si>
-    <t>/history</t>
+    <t>User, Admin</t>
+  </si>
+  <si>
+    <t>getProfile</t>
+  </si>
+  <si>
+    <t>routes/user.js</t>
+  </si>
+  <si>
+    <t>/api/admin/system-logs</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>getLogs</t>
+  </si>
+  <si>
+    <t>routes/admin.js</t>
+  </si>
+  <si>
+    <t>/api/health</t>
+  </si>
+  <si>
+    <t>healthCheck</t>
+  </si>
+  <si>
+    <t>routes/index.js</t>
   </si>
 </sst>
 </file>
@@ -456,16 +474,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -478,187 +496,131 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>7</v>
       </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>13</v>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>